<commit_message>
Atualiza artefatos iGovTI 2026 para respostas 20260621 e ajusta pipeline de avaliacao/consolidacao de evidencias
- Gera e adiciona workbooks iGovTI 2026 com prefixo 20260621 (oficial, comparavel,
  contexto de relatorios, memoria de calculo e comparacao 2023-2026).
- Atualiza mapa de verificacao/achados e resultado da auditoria para fonte 20260621.
- Remove artefatos obsoletos do prefixo 20260611 e prompts conservadores nao mais usados.
- Adiciona scripts de automacao: gerar_igovti.py, atualizar_conjunto_igovti.py,
  run_avaliacao_evidencias.py, run_consolida_avaliacoes.py, verificar_cobertura_achados.py.
- Ajusta pipeline de avaliacao para deduplicacao por orgao e suporte a auditados
  com nomes compostos (separador por virgula).
- Corrige consolidacao de pareceres para nao bloquear PDFs sem texto extraivel
  quando houver upload nativo disponivel.
- Corrige wildcard no script run_consolida_avaliacoes.sh.
</commit_message>
<xml_diff>
--- a/02-Execucao/01-Questionario/Evidencias_Coletadas/urls_anexos_limesurvey_consolidado.xlsx
+++ b/02-Execucao/01-Questionario/Evidencias_Coletadas/urls_anexos_limesurvey_consolidado.xlsx
@@ -1480,7 +1480,7 @@
     <t>CEDAE</t>
   </si>
   <si>
-    <t xml:space="preserve">16.06.2026 17:15:57</t>
+    <t xml:space="preserve">17.06.2026 11:55:48</t>
   </si>
   <si>
     <t>https://www.tcerj.tc.br/limesurvey-novo/index.php/admin/responses/sa/actionDownloadfiles/surveyid/585912/sResponseId/102</t>
@@ -1807,7 +1807,7 @@
     <t xml:space="preserve">CAMPOS DOS GOYTACAZES</t>
   </si>
   <si>
-    <t xml:space="preserve">08.06.2026 16:58:08</t>
+    <t xml:space="preserve">17.06.2026 16:57:00</t>
   </si>
   <si>
     <t>https://www.tcerj.tc.br/limesurvey-novo/index.php/admin/responses/sa/actionDownloadfiles/surveyid/585912/sResponseId/125</t>
@@ -1848,8 +1848,11 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2404,7 +2407,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
+  <cols>
+    <col bestFit="1" min="3" max="3" width="17.125"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
@@ -4316,8 +4322,8 @@
       <c r="C96" t="s">
         <v>480</v>
       </c>
-      <c r="D96" t="s">
-        <v>85</v>
+      <c r="D96" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="E96" t="s">
         <v>481</v>
@@ -4756,8 +4762,8 @@
       <c r="C118" t="s">
         <v>589</v>
       </c>
-      <c r="D118" t="s">
-        <v>85</v>
+      <c r="D118" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="E118" t="s">
         <v>590</v>

</xml_diff>